<commit_message>
data: hourly update 2026-07-18 18:14Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-18.xlsx
+++ b/data/output/workbook/2026-07-18.xlsx
@@ -491,7 +491,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10715625"/>
+    <ext cx="10125075" cy="10887075"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:01</t>
+          <t>2026-07-18 14:13</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q82"/>
+  <dimension ref="A1:Q83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3031,250 +3031,171 @@
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="29" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="29" t="inlineStr">
         <is>
           <t>Chicago White Sox offense vs Toronto Blue Jays defense</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="30" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B69" s="30" t="inlineStr">
+      <c r="B70" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C69" s="30" t="inlineStr">
+      <c r="C70" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D69" s="30" t="inlineStr">
+      <c r="D70" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E69" s="30" t="inlineStr">
+      <c r="E70" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F69" s="30" t="inlineStr">
+      <c r="F70" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G69" s="30" t="inlineStr">
+      <c r="G70" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H69" s="30" t="inlineStr">
+      <c r="H70" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I69" s="30" t="inlineStr">
+      <c r="I70" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J69" s="30" t="inlineStr">
+      <c r="J70" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K69" s="30" t="inlineStr">
+      <c r="K70" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L69" s="30" t="inlineStr">
+      <c r="L70" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M69" s="30" t="inlineStr">
+      <c r="M70" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N69" s="30" t="inlineStr">
+      <c r="N70" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O69" s="30" t="inlineStr">
+      <c r="O70" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P69" s="30" t="inlineStr">
+      <c r="P70" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q69" s="30" t="inlineStr">
+      <c r="Q70" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B70" s="32" t="n">
-        <v>4.953</v>
-      </c>
-      <c r="C70" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="D70" s="32" t="n">
-        <v>5.65</v>
-      </c>
-      <c r="E70" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="F70" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="G70" s="32" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="H70" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I70" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J70" s="36" t="inlineStr">
-        <is>
-          <t>27th</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="L70" s="32" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="M70" s="32" t="n">
-        <v>4.867</v>
-      </c>
-      <c r="N70" s="32" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="O70" s="32" t="n">
-        <v>4.967</v>
-      </c>
-      <c r="P70" s="32" t="n">
-        <v>4.571</v>
-      </c>
-      <c r="Q70" s="34" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>7.792</v>
-      </c>
-      <c r="C71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I71" s="32" t="inlineStr"/>
-      <c r="J71" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>4.953</v>
+      </c>
+      <c r="C71" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" s="32" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="E71" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F71" s="32" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G71" s="32" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H71" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J71" s="36" t="inlineStr">
+        <is>
+          <t>27th</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L71" s="32" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="M71" s="32" t="n">
+        <v>4.867</v>
+      </c>
+      <c r="N71" s="32" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="O71" s="32" t="n">
+        <v>4.967</v>
       </c>
       <c r="P71" s="32" t="n">
-        <v>7.894</v>
+        <v>4.571</v>
       </c>
       <c r="Q71" s="34" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>1.354</v>
+        <v>7.792</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -3338,22 +3259,22 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>0.979</v>
+        <v>7.894</v>
       </c>
       <c r="Q72" s="34" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B73" s="32" t="n">
-        <v>9.208</v>
+        <v>1.354</v>
       </c>
       <c r="C73" s="32" t="inlineStr">
         <is>
@@ -3417,317 +3338,317 @@
         </is>
       </c>
       <c r="P73" s="32" t="n">
-        <v>9.489000000000001</v>
+        <v>0.979</v>
       </c>
       <c r="Q73" s="34" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="31" t="inlineStr">
         <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B74" s="32" t="n">
+        <v>9.208</v>
+      </c>
+      <c r="C74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P74" s="32" t="n">
+        <v>9.489000000000001</v>
+      </c>
+      <c r="Q74" s="34" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B74" s="32" t="n">
+      <c r="B75" s="32" t="n">
         <v>0.627</v>
       </c>
-      <c r="C74" s="32" t="n">
+      <c r="C75" s="32" t="n">
         <v>0.5669999999999999</v>
       </c>
-      <c r="D74" s="32" t="n">
+      <c r="D75" s="32" t="n">
         <v>0.65</v>
       </c>
-      <c r="E74" s="32" t="n">
+      <c r="E75" s="32" t="n">
         <v>0.867</v>
       </c>
-      <c r="F74" s="32" t="n">
+      <c r="F75" s="32" t="n">
         <v>0.9</v>
       </c>
-      <c r="G74" s="32" t="n">
+      <c r="G75" s="32" t="n">
         <v>1.2</v>
       </c>
-      <c r="H74" s="33" t="inlineStr">
+      <c r="H75" s="33" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="I74" s="32" t="inlineStr">
+      <c r="I75" s="32" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="J74" s="36" t="inlineStr">
+      <c r="J75" s="36" t="inlineStr">
         <is>
           <t>28th</t>
         </is>
       </c>
-      <c r="K74" s="32" t="n">
+      <c r="K75" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="L74" s="32" t="n">
+      <c r="L75" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="M74" s="32" t="n">
+      <c r="M75" s="32" t="n">
         <v>0.467</v>
       </c>
-      <c r="N74" s="32" t="n">
+      <c r="N75" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="O74" s="32" t="n">
+      <c r="O75" s="32" t="n">
         <v>0.767</v>
       </c>
-      <c r="P74" s="32" t="n">
+      <c r="P75" s="32" t="n">
         <v>0.554</v>
       </c>
-      <c r="Q74" s="34" t="inlineStr">
+      <c r="Q75" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="29" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>Toronto Blue Jays offense vs Chicago White Sox defense</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="30" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B77" s="30" t="inlineStr">
+      <c r="B78" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C77" s="30" t="inlineStr">
+      <c r="C78" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D77" s="30" t="inlineStr">
+      <c r="D78" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E77" s="30" t="inlineStr">
+      <c r="E78" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F77" s="30" t="inlineStr">
+      <c r="F78" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G77" s="30" t="inlineStr">
+      <c r="G78" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H77" s="30" t="inlineStr">
+      <c r="H78" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I77" s="30" t="inlineStr">
+      <c r="I78" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J77" s="30" t="inlineStr">
+      <c r="J78" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K77" s="30" t="inlineStr">
+      <c r="K78" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L77" s="30" t="inlineStr">
+      <c r="L78" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M77" s="30" t="inlineStr">
+      <c r="M78" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N77" s="30" t="inlineStr">
+      <c r="N78" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O77" s="30" t="inlineStr">
+      <c r="O78" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P77" s="30" t="inlineStr">
+      <c r="P78" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q77" s="30" t="inlineStr">
+      <c r="Q78" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B78" s="32" t="n">
-        <v>4.083</v>
-      </c>
-      <c r="C78" s="32" t="n">
-        <v>4.067</v>
-      </c>
-      <c r="D78" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="E78" s="32" t="n">
-        <v>3.933</v>
-      </c>
-      <c r="F78" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G78" s="32" t="n">
-        <v>6</v>
-      </c>
-      <c r="H78" s="33" t="inlineStr">
-        <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="I78" s="32" t="inlineStr"/>
-      <c r="J78" s="33" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="L78" s="32" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="M78" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="N78" s="32" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="O78" s="32" t="n">
-        <v>3.867</v>
-      </c>
-      <c r="P78" s="32" t="n">
-        <v>4.553</v>
-      </c>
-      <c r="Q78" s="34" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>8.468</v>
-      </c>
-      <c r="C79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>4.083</v>
+      </c>
+      <c r="C79" s="32" t="n">
+        <v>4.067</v>
+      </c>
+      <c r="D79" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E79" s="32" t="n">
+        <v>3.933</v>
+      </c>
+      <c r="F79" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G79" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H79" s="33" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J79" s="33" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L79" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M79" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N79" s="32" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="O79" s="32" t="n">
+        <v>3.867</v>
       </c>
       <c r="P79" s="32" t="n">
-        <v>7.854</v>
+        <v>4.553</v>
       </c>
       <c r="Q79" s="34" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>0.915</v>
+        <v>8.468</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -3791,22 +3712,22 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>1.062</v>
+        <v>7.854</v>
       </c>
       <c r="Q80" s="34" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>7.298</v>
+        <v>0.915</v>
       </c>
       <c r="C81" s="32" t="inlineStr">
         <is>
@@ -3870,72 +3791,151 @@
         </is>
       </c>
       <c r="P81" s="32" t="n">
-        <v>7.938</v>
+        <v>1.062</v>
       </c>
       <c r="Q81" s="34" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
         <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B82" s="32" t="n">
+        <v>7.298</v>
+      </c>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P82" s="32" t="n">
+        <v>7.938</v>
+      </c>
+      <c r="Q82" s="34" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B82" s="32" t="n">
+      <c r="B83" s="32" t="n">
         <v>0.458</v>
       </c>
-      <c r="C82" s="32" t="n">
+      <c r="C83" s="32" t="n">
         <v>0.433</v>
       </c>
-      <c r="D82" s="32" t="n">
+      <c r="D83" s="32" t="n">
         <v>0.45</v>
       </c>
-      <c r="E82" s="32" t="n">
+      <c r="E83" s="32" t="n">
         <v>0.533</v>
       </c>
-      <c r="F82" s="32" t="n">
+      <c r="F83" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="G82" s="32" t="n">
+      <c r="G83" s="32" t="n">
         <v>1.2</v>
       </c>
-      <c r="H82" s="33" t="inlineStr">
+      <c r="H83" s="33" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="I82" s="32" t="inlineStr">
+      <c r="I83" s="32" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="J82" s="33" t="inlineStr">
+      <c r="J83" s="33" t="inlineStr">
         <is>
           <t>8th</t>
         </is>
       </c>
-      <c r="K82" s="32" t="n">
+      <c r="K83" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="L82" s="32" t="n">
+      <c r="L83" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="M82" s="32" t="n">
+      <c r="M83" s="32" t="n">
         <v>0.467</v>
       </c>
-      <c r="N82" s="32" t="n">
+      <c r="N83" s="32" t="n">
         <v>0.35</v>
       </c>
-      <c r="O82" s="32" t="n">
+      <c r="O83" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="P82" s="32" t="n">
+      <c r="P83" s="32" t="n">
         <v>0.53</v>
       </c>
-      <c r="Q82" s="34" t="inlineStr">
+      <c r="Q83" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -9310,10 +9310,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.605</v>
+        <v>0.6057</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-153</v>
+        <v>-154</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>150</v>
@@ -9340,7 +9340,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 60.5% (fair -153). Your call.</t>
+          <t>Model 60.6% (fair -154). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9895,22 +9895,22 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4162</v>
+        <v>0.5371</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>140</v>
+        <v>-116</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>170</v>
+        <v>112</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9934,7 +9934,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 41.6% (fair +140). Your call.</t>
+          <t>Model 53.7% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9961,22 +9961,22 @@
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5216000000000001</v>
+        <v>0.4137</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-109</v>
+        <v>142</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>112</v>
+        <v>170</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -10000,7 +10000,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 41.4% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10102,10 +10102,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4922</v>
+        <v>0.4945</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>120</v>
@@ -10132,7 +10132,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10432,10 +10432,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.395</v>
+        <v>0.3943</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>168</v>
@@ -10462,7 +10462,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 39.5% (fair +153). Your call.</t>
+          <t>Model 39.4% (fair +154). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12223,10 +12223,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5181</v>
+        <v>0.5151</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-108</v>
+        <v>-106</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>104</v>
@@ -12253,7 +12253,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -108). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12289,10 +12289,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4819</v>
+        <v>0.4849</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-102</v>
@@ -12319,7 +12319,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 48.2% (fair +108). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -12355,10 +12355,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4784</v>
+        <v>0.4629</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>113</v>
@@ -12385,7 +12385,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 46.3% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12421,10 +12421,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5216000000000001</v>
+        <v>0.5371</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-109</v>
+        <v>-116</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>112</v>
@@ -12451,7 +12451,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 53.7% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -12487,10 +12487,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5838</v>
+        <v>0.5863</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-140</v>
+        <v>-142</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>-163</v>
@@ -12517,7 +12517,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 58.4% (fair -140). Your call.</t>
+          <t>Model 58.6% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -12553,10 +12553,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4162</v>
+        <v>0.4137</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>170</v>
@@ -12583,7 +12583,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 41.6% (fair +140). Your call.</t>
+          <t>Model 41.4% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -14995,10 +14995,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.5092</v>
+        <v>0.506</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="H71" s="15" t="n"/>
       <c r="I71" s="13">
@@ -15023,7 +15023,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 50.6% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -15059,10 +15059,10 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.4908</v>
+        <v>0.494</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H72" s="15" t="n"/>
       <c r="I72" s="13">
@@ -15087,7 +15087,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 49.4% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -15383,10 +15383,10 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.4807</v>
+        <v>0.4868</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H77" s="15" t="n"/>
       <c r="I77" s="13">
@@ -15411,7 +15411,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -15447,10 +15447,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.5193</v>
+        <v>0.5132</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="H78" s="15" t="n"/>
       <c r="I78" s="13">
@@ -15475,7 +15475,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -16295,10 +16295,10 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.4916</v>
+        <v>0.4868</v>
       </c>
       <c r="G91" s="14" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H91" s="15" t="n">
         <v>102</v>
@@ -16325,7 +16325,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -16361,10 +16361,10 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.5084</v>
+        <v>0.5132</v>
       </c>
       <c r="G92" s="14" t="n">
-        <v>-103</v>
+        <v>-105</v>
       </c>
       <c r="H92" s="15" t="n">
         <v>-105</v>
@@ -16391,7 +16391,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -16427,10 +16427,10 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.395</v>
+        <v>0.3943</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H93" s="15" t="n">
         <v>168</v>
@@ -16457,7 +16457,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 39.5% (fair +153). Your call.</t>
+          <t>Model 39.4% (fair +154). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -16493,10 +16493,10 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.605</v>
+        <v>0.6057</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>-153</v>
+        <v>-154</v>
       </c>
       <c r="H94" s="15" t="n">
         <v>150</v>
@@ -16523,7 +16523,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 60.5% (fair -153). Your call.</t>
+          <t>Model 60.6% (fair -154). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -16559,10 +16559,10 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>0.4938</v>
+        <v>0.495</v>
       </c>
       <c r="G95" s="14" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H95" s="15" t="n">
         <v>-104</v>
@@ -16589,7 +16589,7 @@
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +103). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O95" s="15" t="n"/>
@@ -16625,10 +16625,10 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.5062</v>
+        <v>0.505</v>
       </c>
       <c r="G96" s="14" t="n">
-        <v>-103</v>
+        <v>-102</v>
       </c>
       <c r="H96" s="15" t="n">
         <v>108</v>
@@ -16655,7 +16655,7 @@
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -103). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O96" s="15" t="n"/>
@@ -16691,10 +16691,10 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.5376</v>
+        <v>0.5281</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>-116</v>
+        <v>-112</v>
       </c>
       <c r="H97" s="15" t="n">
         <v>-120</v>
@@ -16721,7 +16721,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -116). Your call.</t>
+          <t>Model 52.8% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16757,10 +16757,10 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.4624</v>
+        <v>0.4719</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H98" s="15" t="n">
         <v>100</v>
@@ -16787,7 +16787,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 47.2% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16823,7 +16823,7 @@
         </is>
       </c>
       <c r="F99" s="13" t="n">
-        <v>0.5895</v>
+        <v>0.59</v>
       </c>
       <c r="G99" s="14" t="n">
         <v>-144</v>
@@ -16889,7 +16889,7 @@
         </is>
       </c>
       <c r="F100" s="13" t="n">
-        <v>0.4105</v>
+        <v>0.41</v>
       </c>
       <c r="G100" s="14" t="n">
         <v>144</v>
@@ -18011,10 +18011,10 @@
         </is>
       </c>
       <c r="F117" s="13" t="n">
-        <v>0.4876</v>
+        <v>0.5078</v>
       </c>
       <c r="G117" s="14" t="n">
-        <v>105</v>
+        <v>-103</v>
       </c>
       <c r="H117" s="15" t="n">
         <v>100</v>
@@ -18041,7 +18041,7 @@
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O117" s="15" t="n"/>
@@ -18077,10 +18077,10 @@
         </is>
       </c>
       <c r="F118" s="13" t="n">
-        <v>0.5124</v>
+        <v>0.4922</v>
       </c>
       <c r="G118" s="14" t="n">
-        <v>-105</v>
+        <v>103</v>
       </c>
       <c r="H118" s="15" t="n">
         <v>-105</v>
@@ -18107,7 +18107,7 @@
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O118" s="15" t="n"/>
@@ -18143,7 +18143,7 @@
         </is>
       </c>
       <c r="F119" s="13" t="n">
-        <v>0.3994</v>
+        <v>0.3995</v>
       </c>
       <c r="G119" s="14" t="n">
         <v>150</v>
@@ -18173,7 +18173,7 @@
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +150). Your call.</t>
+          <t>Model 40.0% (fair +150). Your call.</t>
         </is>
       </c>
       <c r="O119" s="15" t="n"/>
@@ -18209,7 +18209,7 @@
         </is>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.6006</v>
+        <v>0.6005</v>
       </c>
       <c r="G120" s="14" t="n">
         <v>-150</v>
@@ -18275,7 +18275,7 @@
         </is>
       </c>
       <c r="F121" s="13" t="n">
-        <v>0.4466</v>
+        <v>0.446</v>
       </c>
       <c r="G121" s="14" t="n">
         <v>124</v>
@@ -18305,7 +18305,7 @@
       </c>
       <c r="N121" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 44.6% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O121" s="15" t="n"/>
@@ -18341,7 +18341,7 @@
         </is>
       </c>
       <c r="F122" s="13" t="n">
-        <v>0.5534</v>
+        <v>0.554</v>
       </c>
       <c r="G122" s="14" t="n">
         <v>-124</v>
@@ -18371,7 +18371,7 @@
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 55.4% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O122" s="15" t="n"/>
@@ -18407,10 +18407,10 @@
         </is>
       </c>
       <c r="F123" s="13" t="n">
-        <v>0.4905</v>
+        <v>0.4965</v>
       </c>
       <c r="G123" s="14" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H123" s="15" t="n">
         <v>100</v>
@@ -18437,7 +18437,7 @@
       </c>
       <c r="N123" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 49.6% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O123" s="15" t="n"/>
@@ -18473,10 +18473,10 @@
         </is>
       </c>
       <c r="F124" s="13" t="n">
-        <v>0.5095000000000001</v>
+        <v>0.5035000000000001</v>
       </c>
       <c r="G124" s="14" t="n">
-        <v>-104</v>
+        <v>-101</v>
       </c>
       <c r="H124" s="15" t="n">
         <v>-110</v>
@@ -18503,7 +18503,7 @@
       </c>
       <c r="N124" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 50.4% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O124" s="15" t="n"/>
@@ -18539,10 +18539,10 @@
         </is>
       </c>
       <c r="F125" s="13" t="n">
-        <v>0.3633</v>
+        <v>0.365</v>
       </c>
       <c r="G125" s="14" t="n">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H125" s="15" t="n">
         <v>168</v>
@@ -18569,7 +18569,7 @@
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>Model 36.3% (fair +175). Your call.</t>
+          <t>Model 36.5% (fair +174). Your call.</t>
         </is>
       </c>
       <c r="O125" s="15" t="n"/>
@@ -18605,10 +18605,10 @@
         </is>
       </c>
       <c r="F126" s="13" t="n">
-        <v>0.6367</v>
+        <v>0.635</v>
       </c>
       <c r="G126" s="14" t="n">
-        <v>-175</v>
+        <v>-174</v>
       </c>
       <c r="H126" s="15" t="n">
         <v>-190</v>
@@ -18635,7 +18635,7 @@
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>Model 63.7% (fair -175). Your call.</t>
+          <t>Model 63.5% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O126" s="15" t="n"/>
@@ -19067,10 +19067,10 @@
         </is>
       </c>
       <c r="F133" s="13" t="n">
-        <v>0.5078</v>
+        <v>0.5055000000000001</v>
       </c>
       <c r="G133" s="14" t="n">
-        <v>-103</v>
+        <v>-102</v>
       </c>
       <c r="H133" s="15" t="n">
         <v>-122</v>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="N133" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 50.6% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O133" s="15" t="n"/>
@@ -19133,10 +19133,10 @@
         </is>
       </c>
       <c r="F134" s="13" t="n">
-        <v>0.4922</v>
+        <v>0.4945</v>
       </c>
       <c r="G134" s="14" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H134" s="15" t="n">
         <v>120</v>
@@ -19163,7 +19163,7 @@
       </c>
       <c r="N134" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O134" s="15" t="n"/>
@@ -19199,10 +19199,10 @@
         </is>
       </c>
       <c r="F135" s="13" t="n">
-        <v>0.491</v>
+        <v>0.4693</v>
       </c>
       <c r="G135" s="14" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="H135" s="15" t="n">
         <v>100</v>
@@ -19229,7 +19229,7 @@
       </c>
       <c r="N135" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 46.9% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O135" s="15" t="n"/>
@@ -19265,10 +19265,10 @@
         </is>
       </c>
       <c r="F136" s="13" t="n">
-        <v>0.509</v>
+        <v>0.5306999999999999</v>
       </c>
       <c r="G136" s="14" t="n">
-        <v>-104</v>
+        <v>-113</v>
       </c>
       <c r="H136" s="15" t="n">
         <v>-105</v>
@@ -19295,7 +19295,7 @@
       </c>
       <c r="N136" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O136" s="15" t="n"/>
@@ -19331,10 +19331,10 @@
         </is>
       </c>
       <c r="F137" s="13" t="n">
-        <v>0.5669</v>
+        <v>0.5686</v>
       </c>
       <c r="G137" s="14" t="n">
-        <v>-131</v>
+        <v>-132</v>
       </c>
       <c r="H137" s="15" t="n">
         <v>-125</v>
@@ -19361,7 +19361,7 @@
       </c>
       <c r="N137" s="19" t="inlineStr">
         <is>
-          <t>Model 56.7% (fair -131). Your call.</t>
+          <t>Model 56.9% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O137" s="15" t="n"/>
@@ -19397,10 +19397,10 @@
         </is>
       </c>
       <c r="F138" s="13" t="n">
-        <v>0.4331</v>
+        <v>0.4314</v>
       </c>
       <c r="G138" s="14" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H138" s="15" t="n">
         <v>105</v>
@@ -19427,7 +19427,7 @@
       </c>
       <c r="N138" s="19" t="inlineStr">
         <is>
-          <t>Model 43.3% (fair +131). Your call.</t>
+          <t>Model 43.1% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O138" s="15" t="n"/>
@@ -19983,10 +19983,10 @@
         </is>
       </c>
       <c r="F147" s="13" t="n">
-        <v>0.4293</v>
+        <v>0.4244</v>
       </c>
       <c r="G147" s="14" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H147" s="15" t="n"/>
       <c r="I147" s="13">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="N147" s="19" t="inlineStr">
         <is>
-          <t>Model 42.9% (fair +133). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O147" s="15" t="n"/>
@@ -20047,10 +20047,10 @@
         </is>
       </c>
       <c r="F148" s="13" t="n">
-        <v>0.5707</v>
+        <v>0.5756</v>
       </c>
       <c r="G148" s="14" t="n">
-        <v>-133</v>
+        <v>-136</v>
       </c>
       <c r="H148" s="15" t="n"/>
       <c r="I148" s="13">
@@ -20075,7 +20075,7 @@
       </c>
       <c r="N148" s="19" t="inlineStr">
         <is>
-          <t>Model 57.1% (fair -133). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O148" s="15" t="n"/>
@@ -20239,10 +20239,10 @@
         </is>
       </c>
       <c r="F151" s="13" t="n">
-        <v>0.4786</v>
+        <v>0.4802</v>
       </c>
       <c r="G151" s="14" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H151" s="15" t="n"/>
       <c r="I151" s="13">
@@ -20267,7 +20267,7 @@
       </c>
       <c r="N151" s="19" t="inlineStr">
         <is>
-          <t>Model 47.9% (fair +109). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O151" s="15" t="n"/>
@@ -20303,10 +20303,10 @@
         </is>
       </c>
       <c r="F152" s="13" t="n">
-        <v>0.5214</v>
+        <v>0.5198</v>
       </c>
       <c r="G152" s="14" t="n">
-        <v>-109</v>
+        <v>-108</v>
       </c>
       <c r="H152" s="15" t="n"/>
       <c r="I152" s="13">
@@ -20331,7 +20331,7 @@
       </c>
       <c r="N152" s="19" t="inlineStr">
         <is>
-          <t>Model 52.1% (fair -109). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O152" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-18 23:03Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-18.xlsx
+++ b/data/output/workbook/2026-07-18.xlsx
@@ -551,7 +551,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10915650"/>
+    <ext cx="10125075" cy="10648950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:03</t>
+          <t>2026-07-18 19:02</t>
         </is>
       </c>
     </row>
@@ -4886,7 +4886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q83"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4903,171 +4903,250 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles offense vs Houston Astros defense</t>
+        </is>
+      </c>
+    </row>
     <row r="69">
-      <c r="A69" s="29" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles offense vs Houston Astros defense</t>
+      <c r="A69" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B69" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D69" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E69" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F69" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G69" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H69" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I69" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J69" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K69" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L69" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M69" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N69" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O69" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P69" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q69" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B70" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C70" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D70" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E70" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F70" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G70" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H70" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I70" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J70" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K70" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L70" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M70" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N70" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O70" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P70" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q70" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="n">
+        <v>4.593</v>
+      </c>
+      <c r="C70" s="32" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="D70" s="32" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="E70" s="32" t="n">
+        <v>4.333</v>
+      </c>
+      <c r="F70" s="32" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G70" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="H70" s="33" t="inlineStr">
+        <is>
+          <t>9th</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J70" s="36" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="L70" s="32" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M70" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="N70" s="32" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="O70" s="32" t="n">
+        <v>4.967</v>
+      </c>
+      <c r="P70" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q70" s="34" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>4.593</v>
-      </c>
-      <c r="C71" s="32" t="n">
-        <v>4.433</v>
-      </c>
-      <c r="D71" s="32" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="E71" s="32" t="n">
-        <v>4.333</v>
-      </c>
-      <c r="F71" s="32" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="G71" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="H71" s="33" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="I71" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J71" s="36" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="L71" s="32" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="M71" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="N71" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="O71" s="32" t="n">
-        <v>4.967</v>
+        <v>8.208</v>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr"/>
+      <c r="J71" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P71" s="32" t="n">
-        <v>5</v>
+        <v>7.625</v>
       </c>
       <c r="Q71" s="34" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>8.208</v>
+        <v>1.271</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -5131,22 +5210,22 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>7.625</v>
+        <v>1.292</v>
       </c>
       <c r="Q72" s="34" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B73" s="32" t="n">
-        <v>1.271</v>
+        <v>8.917</v>
       </c>
       <c r="C73" s="32" t="inlineStr">
         <is>
@@ -5210,313 +5289,313 @@
         </is>
       </c>
       <c r="P73" s="32" t="n">
-        <v>1.292</v>
+        <v>8.417</v>
       </c>
       <c r="Q73" s="34" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B74" s="32" t="n">
-        <v>8.917</v>
-      </c>
-      <c r="C74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>0.482</v>
+      </c>
+      <c r="C74" s="32" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="D74" s="32" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E74" s="32" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="F74" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G74" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="36" t="inlineStr">
+        <is>
+          <t>28th</t>
         </is>
       </c>
       <c r="I74" s="32" t="inlineStr"/>
-      <c r="J74" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J74" s="35" t="inlineStr">
+        <is>
+          <t>17th</t>
+        </is>
+      </c>
+      <c r="K74" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L74" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M74" s="32" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="N74" s="32" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="O74" s="32" t="n">
+        <v>0.667</v>
       </c>
       <c r="P74" s="32" t="n">
-        <v>8.417</v>
+        <v>0.635</v>
       </c>
       <c r="Q74" s="34" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B75" s="32" t="n">
-        <v>0.482</v>
-      </c>
-      <c r="C75" s="32" t="n">
-        <v>0.5669999999999999</v>
-      </c>
-      <c r="D75" s="32" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E75" s="32" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="F75" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G75" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="36" t="inlineStr">
-        <is>
-          <t>28th</t>
-        </is>
-      </c>
-      <c r="I75" s="32" t="inlineStr"/>
-      <c r="J75" s="35" t="inlineStr">
-        <is>
-          <t>17th</t>
-        </is>
-      </c>
-      <c r="K75" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="L75" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M75" s="32" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="N75" s="32" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="O75" s="32" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="P75" s="32" t="n">
-        <v>0.635</v>
-      </c>
-      <c r="Q75" s="34" t="inlineStr">
-        <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>Houston Astros offense vs Baltimore Orioles defense</t>
+        </is>
+      </c>
+    </row>
     <row r="77">
-      <c r="A77" s="29" t="inlineStr">
-        <is>
-          <t>Houston Astros offense vs Baltimore Orioles defense</t>
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E77" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F77" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H77" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I77" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J77" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K77" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L77" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M77" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N77" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O77" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P77" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q77" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B78" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C78" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E78" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F78" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G78" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H78" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I78" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J78" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K78" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L78" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M78" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N78" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O78" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P78" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q78" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A78" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B78" s="32" t="n">
+        <v>4.885</v>
+      </c>
+      <c r="C78" s="32" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D78" s="32" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E78" s="32" t="n">
+        <v>5.267</v>
+      </c>
+      <c r="F78" s="32" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G78" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H78" s="35" t="inlineStr">
+        <is>
+          <t>15th</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr"/>
+      <c r="J78" s="33" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L78" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M78" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="N78" s="32" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="O78" s="32" t="n">
+        <v>3.867</v>
+      </c>
+      <c r="P78" s="32" t="n">
+        <v>4.686</v>
+      </c>
+      <c r="Q78" s="34" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>4.885</v>
-      </c>
-      <c r="C79" s="32" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="D79" s="32" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="E79" s="32" t="n">
-        <v>5.267</v>
-      </c>
-      <c r="F79" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="G79" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="H79" s="35" t="inlineStr">
-        <is>
-          <t>15th</t>
+        <v>8.083</v>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="33" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="L79" s="32" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="M79" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="N79" s="32" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="O79" s="32" t="n">
-        <v>3.867</v>
+      <c r="J79" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P79" s="32" t="n">
-        <v>4.686</v>
+        <v>8.833</v>
       </c>
       <c r="Q79" s="34" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>8.083</v>
+        <v>1.417</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -5580,22 +5659,22 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>8.833</v>
+        <v>1.062</v>
       </c>
       <c r="Q80" s="34" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>1.417</v>
+        <v>7.729</v>
       </c>
       <c r="C81" s="32" t="inlineStr">
         <is>
@@ -5659,147 +5738,68 @@
         </is>
       </c>
       <c r="P81" s="32" t="n">
-        <v>1.062</v>
+        <v>8</v>
       </c>
       <c r="Q81" s="34" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B82" s="32" t="n">
-        <v>7.729</v>
-      </c>
-      <c r="C82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H82" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="C82" s="32" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D82" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E82" s="32" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="F82" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G82" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H82" s="33" t="inlineStr">
+        <is>
+          <t>9th</t>
         </is>
       </c>
       <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J82" s="35" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="K82" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L82" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M82" s="32" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="N82" s="32" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="O82" s="32" t="n">
+        <v>0.667</v>
       </c>
       <c r="P82" s="32" t="n">
-        <v>8</v>
+        <v>0.459</v>
       </c>
       <c r="Q82" s="34" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B83" s="32" t="n">
-        <v>0.6820000000000001</v>
-      </c>
-      <c r="C83" s="32" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D83" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E83" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="F83" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G83" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H83" s="33" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="I83" s="32" t="inlineStr"/>
-      <c r="J83" s="35" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="K83" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L83" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M83" s="32" t="n">
-        <v>0.267</v>
-      </c>
-      <c r="N83" s="32" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="O83" s="32" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="P83" s="32" t="n">
-        <v>0.459</v>
-      </c>
-      <c r="Q83" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8848,10 +8848,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.7046</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-239</v>
+        <v>-238</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>178</v>
@@ -8878,7 +8878,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 70.5% (fair -239). Your call.</t>
+          <t>Model 70.4% (fair -238). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8890,17 +8890,17 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -8910,14 +8910,14 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles +1.5</t>
+          <t>Pittsburgh Pirates +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6751</v>
+        <v>0.6687000000000001</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-208</v>
+        <v>-202</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>178</v>
@@ -8944,7 +8944,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 67.5% (fair -208). Your call.</t>
+          <t>Model 66.9% (fair -202). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8956,17 +8956,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8976,17 +8976,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates +1.5</t>
+          <t>Baltimore Orioles +1.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6687000000000001</v>
+        <v>0.6751</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-202</v>
+        <v>-208</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -9010,7 +9010,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 66.9% (fair -202). Your call.</t>
+          <t>Model 67.5% (fair -208). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9112,10 +9112,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.6541</v>
+        <v>0.6585</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-189</v>
+        <v>-193</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>167</v>
@@ -9142,7 +9142,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 65.4% (fair -189). Your call.</t>
+          <t>Model 65.8% (fair -193). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9178,10 +9178,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6386000000000001</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-177</v>
+        <v>-175</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>167</v>
@@ -9208,7 +9208,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 63.9% (fair -177). Your call.</t>
+          <t>Model 63.7% (fair -175). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9442,10 +9442,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.6447000000000001</v>
+        <v>0.6381</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-181</v>
+        <v>-176</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>113</v>
@@ -9472,7 +9472,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 64.5% (fair -181). Your call.</t>
+          <t>Model 63.8% (fair -176). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9489,12 +9489,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>23:20</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -9504,17 +9504,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.6089</v>
+        <v>0.646</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-156</v>
+        <v>-182</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9538,7 +9538,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 64.6% (fair -182). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9550,17 +9550,17 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>23:20</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -9570,17 +9570,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6228</v>
+        <v>0.5989</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-165</v>
+        <v>-149</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9604,7 +9604,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 62.3% (fair -165). Your call.</t>
+          <t>Model 59.9% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9621,12 +9621,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -9636,14 +9636,14 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.6114999999999999</v>
+        <v>0.6228</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-157</v>
+        <v>-165</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>102</v>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 61.1% (fair -157). Your call.</t>
+          <t>Model 62.3% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -9706,10 +9706,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.6112</v>
+        <v>0.6179</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-157</v>
+        <v>-162</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>102</v>
@@ -9736,7 +9736,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 61.1% (fair -157). Your call.</t>
+          <t>Model 61.8% (fair -162). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -9768,17 +9768,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Under 11</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5912000000000001</v>
+        <v>0.6114999999999999</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-145</v>
+        <v>-157</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 59.1% (fair -145). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9814,17 +9814,17 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9834,17 +9834,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 11</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5631</v>
+        <v>0.5862000000000001</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-129</v>
+        <v>-142</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9868,7 +9868,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 58.6% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9885,12 +9885,12 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -9900,17 +9900,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5898</v>
+        <v>0.5516</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-144</v>
+        <v>-123</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9934,7 +9934,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9946,17 +9946,17 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Minnesota Lynx</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -9966,14 +9966,14 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 165.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5867</v>
+        <v>0.5886</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-142</v>
+        <v>-143</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>100</v>
@@ -10000,7 +10000,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10012,17 +10012,17 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Atlanta Dream</t>
+          <t>Portland Fire @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -10032,17 +10032,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 173.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5629</v>
+        <v>0.5879</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-129</v>
+        <v>-143</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>108</v>
+        <v>-102</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 58.8% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10078,37 +10078,37 @@
     <row r="24">
       <c r="A24" s="20" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Indiana Fever</t>
+          <t>Chicago Sky @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Chicago Sky +10.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5296999999999999</v>
+        <v>0.5403</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-113</v>
+        <v>-118</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10132,7 +10132,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10168,10 +10168,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5332</v>
+        <v>0.5287999999999999</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-114</v>
+        <v>-112</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>117</v>
@@ -10198,7 +10198,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10210,37 +10210,37 @@
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Atlanta Dream</t>
+          <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky +10.5</t>
+          <t>Over 148.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5415</v>
+        <v>0.5705</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-118</v>
+        <v>-133</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10264,7 +10264,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10281,12 +10281,12 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Golden State Valkyries</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -10296,17 +10296,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Over 148.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5693</v>
+        <v>0.4945</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-132</v>
+        <v>102</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -10330,7 +10330,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10347,32 +10347,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>New York Liberty @ Indiana Fever</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4931</v>
+        <v>0.5359</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>103</v>
+        <v>-115</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10396,7 +10396,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -11167,10 +11167,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.6112</v>
+        <v>0.6179</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-157</v>
+        <v>-162</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>102</v>
@@ -11197,7 +11197,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 61.1% (fair -157). Your call.</t>
+          <t>Model 61.8% (fair -162). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -11233,10 +11233,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3888</v>
+        <v>0.3821</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>128</v>
@@ -11263,7 +11263,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 38.9% (fair +157). Your call.</t>
+          <t>Model 38.2% (fair +162). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -11299,10 +11299,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.2954</v>
+        <v>0.2959</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>175</v>
@@ -11329,7 +11329,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 29.5% (fair +239). Your call.</t>
+          <t>Model 29.6% (fair +238). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -11365,10 +11365,10 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.7046</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-239</v>
+        <v>-238</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>178</v>
@@ -11395,7 +11395,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 70.5% (fair -239). Your call.</t>
+          <t>Model 70.4% (fair -238). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -11563,10 +11563,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4931</v>
+        <v>0.4945</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>130</v>
@@ -11593,7 +11593,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -11629,10 +11629,10 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4198</v>
+        <v>0.4185000000000001</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>-104</v>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 41.9% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -11695,7 +11695,7 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4017</v>
+        <v>0.4011</v>
       </c>
       <c r="G21" s="14" t="n">
         <v>149</v>
@@ -11725,7 +11725,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 40.2% (fair +149). Your call.</t>
+          <t>Model 40.1% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5983000000000001</v>
+        <v>0.5989</v>
       </c>
       <c r="G22" s="14" t="n">
         <v>-149</v>
@@ -11791,7 +11791,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 59.8% (fair -149). Your call.</t>
+          <t>Model 59.9% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -11827,10 +11827,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.2811455999999998</v>
+        <v>0.25926</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>256</v>
+        <v>286</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>156</v>
@@ -11857,7 +11857,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 28.1% (fair +256). Your call.</t>
+          <t>Model 25.9% (fair +286). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -11893,10 +11893,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.7188544000000002</v>
+        <v>0.74074</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-256</v>
+        <v>-286</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>-130</v>
@@ -11923,7 +11923,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 71.9% (fair -256). Your call.</t>
+          <t>Model 74.1% (fair -286). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11959,10 +11959,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.414</v>
+        <v>0.4144</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>103</v>
@@ -11989,7 +11989,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 41.4% (fair +142). Your call.</t>
+          <t>Model 41.4% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -12025,7 +12025,7 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4997000000000001</v>
+        <v>0.4993</v>
       </c>
       <c r="G26" s="14" t="n">
         <v>100</v>
@@ -12055,7 +12055,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair +100). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -12091,10 +12091,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4489</v>
+        <v>0.4509</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>125</v>
@@ -12121,7 +12121,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 44.9% (fair +123). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -12157,10 +12157,10 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5510999999999999</v>
+        <v>0.5490999999999999</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-123</v>
+        <v>-122</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>-127</v>
@@ -12187,7 +12187,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -12223,10 +12223,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5159</v>
+        <v>0.5206</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-107</v>
+        <v>-109</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>102</v>
@@ -12253,7 +12253,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12289,10 +12289,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4841</v>
+        <v>0.4794</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-103</v>
@@ -12319,7 +12319,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -12355,10 +12355,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4762</v>
+        <v>0.4683</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>122</v>
@@ -12385,7 +12385,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12421,10 +12421,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5317000000000001</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-110</v>
+        <v>-114</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -12451,7 +12451,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -12487,10 +12487,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5847</v>
+        <v>0.5838</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-141</v>
+        <v>-140</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>-163</v>
@@ -12517,7 +12517,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 58.4% (fair -140). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -12553,10 +12553,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4153</v>
+        <v>0.4162</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>170</v>
@@ -12583,7 +12583,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 41.6% (fair +140). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -12619,7 +12619,7 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4813</v>
+        <v>0.4815</v>
       </c>
       <c r="G35" s="14" t="n">
         <v>108</v>
@@ -12649,7 +12649,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 48.2% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -12685,7 +12685,7 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5187</v>
+        <v>0.5185</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>-108</v>
@@ -12715,7 +12715,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 51.8% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -12751,7 +12751,7 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4837</v>
+        <v>0.4836</v>
       </c>
       <c r="G37" s="14" t="n">
         <v>107</v>
@@ -12817,7 +12817,7 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5163</v>
+        <v>0.5164</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>-107</v>
@@ -12883,10 +12883,10 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.601</v>
+        <v>0.5988</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-151</v>
+        <v>-149</v>
       </c>
       <c r="H39" s="15" t="n">
         <v>-138</v>
@@ -12913,7 +12913,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 60.1% (fair -151). Your call.</t>
+          <t>Model 59.9% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12949,10 +12949,10 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.399</v>
+        <v>0.4012</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H40" s="15" t="n">
         <v>138</v>
@@ -12979,7 +12979,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +151). Your call.</t>
+          <t>Model 40.1% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -13411,10 +13411,10 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4837</v>
+        <v>0.4805</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H47" s="15" t="n">
         <v>-102</v>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -13477,10 +13477,10 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5163</v>
+        <v>0.5195</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-107</v>
+        <v>-108</v>
       </c>
       <c r="H48" s="15" t="n">
         <v>104</v>
@@ -13507,7 +13507,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -13543,10 +13543,10 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.3349</v>
+        <v>0.3398</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="H49" s="15" t="n">
         <v>108</v>
@@ -13573,7 +13573,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 33.5% (fair +199). Your call.</t>
+          <t>Model 34.0% (fair +194). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -13609,10 +13609,10 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.5912000000000001</v>
+        <v>0.5862000000000001</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-145</v>
+        <v>-142</v>
       </c>
       <c r="H50" s="15" t="n">
         <v>108</v>
@@ -13639,7 +13639,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 59.1% (fair -145). Your call.</t>
+          <t>Model 58.6% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -13675,7 +13675,7 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.612</v>
+        <v>0.6131</v>
       </c>
       <c r="G51" s="14" t="n">
         <v>-158</v>
@@ -13705,7 +13705,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 61.3% (fair -158). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -13741,7 +13741,7 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.388</v>
+        <v>0.3869</v>
       </c>
       <c r="G52" s="14" t="n">
         <v>158</v>
@@ -13771,7 +13771,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 38.7% (fair +158). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -15251,10 +15251,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.2789</v>
+        <v>0.2853</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>109</v>
@@ -15281,7 +15281,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 27.9% (fair +259). Your call.</t>
+          <t>Model 28.5% (fair +251). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -15317,10 +15317,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.6447000000000001</v>
+        <v>0.6381</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-181</v>
+        <v>-176</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>113</v>
@@ -15347,7 +15347,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 64.5% (fair -181). Your call.</t>
+          <t>Model 63.8% (fair -176). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -15383,10 +15383,10 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.4466</v>
+        <v>0.4281</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="H77" s="15" t="n"/>
       <c r="I77" s="13">
@@ -15411,7 +15411,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 42.8% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -15447,10 +15447,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.5534</v>
+        <v>0.5719</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>-124</v>
+        <v>-134</v>
       </c>
       <c r="H78" s="15" t="n"/>
       <c r="I78" s="13">
@@ -15475,7 +15475,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -15511,10 +15511,10 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.5817</v>
+        <v>0.5776</v>
       </c>
       <c r="G79" s="14" t="n">
-        <v>-139</v>
+        <v>-137</v>
       </c>
       <c r="H79" s="15" t="n"/>
       <c r="I79" s="13">
@@ -15539,7 +15539,7 @@
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O79" s="15" t="n"/>
@@ -15575,10 +15575,10 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.4183</v>
+        <v>0.4224</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H80" s="15" t="n"/>
       <c r="I80" s="13">
@@ -15603,7 +15603,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -15639,10 +15639,10 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.4868</v>
+        <v>0.4807</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H81" s="15" t="n"/>
       <c r="I81" s="13">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.1% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -15703,10 +15703,10 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.5132</v>
+        <v>0.5193</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>-105</v>
+        <v>-108</v>
       </c>
       <c r="H82" s="15" t="n"/>
       <c r="I82" s="13">
@@ -15731,7 +15731,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.9% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -15767,7 +15767,7 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.4905</v>
+        <v>0.4903999999999999</v>
       </c>
       <c r="G83" s="14" t="n">
         <v>104</v>
@@ -15797,7 +15797,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15833,7 +15833,7 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.5095</v>
+        <v>0.5096000000000001</v>
       </c>
       <c r="G84" s="14" t="n">
         <v>-104</v>
@@ -15863,7 +15863,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -15899,10 +15899,10 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.4948</v>
+        <v>0.4845</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H85" s="15" t="n">
         <v>113</v>
@@ -15929,7 +15929,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 48.4% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -15965,10 +15965,10 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.5052</v>
+        <v>0.5155000000000001</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>-102</v>
+        <v>-106</v>
       </c>
       <c r="H86" s="15" t="n">
         <v>105</v>
@@ -15995,7 +15995,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 51.6% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -16031,13 +16031,13 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.6165</v>
+        <v>0.623</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>-161</v>
+        <v>-165</v>
       </c>
       <c r="H87" s="15" t="n">
-        <v>-156</v>
+        <v>-163</v>
       </c>
       <c r="I87" s="13">
         <f>IF($H$87="","",IF($H$87&lt;0,-$H$87/(-$H$87+100),100/($H$87+100)))</f>
@@ -16061,7 +16061,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 62.3% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -16097,10 +16097,10 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.3835</v>
+        <v>0.377</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="H88" s="15" t="n">
         <v>178</v>
@@ -16127,7 +16127,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 37.7% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -16163,10 +16163,10 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.4762999999999999</v>
+        <v>0.4778</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H89" s="15" t="n">
         <v>104</v>
@@ -16193,7 +16193,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -16229,13 +16229,13 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.5237000000000001</v>
+        <v>0.5222</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>-110</v>
+        <v>-109</v>
       </c>
       <c r="H90" s="15" t="n">
-        <v>-106</v>
+        <v>-104</v>
       </c>
       <c r="I90" s="13">
         <f>IF($H$90="","",IF($H$90&lt;0,-$H$90/(-$H$90+100),100/($H$90+100)))</f>
@@ -16259,7 +16259,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>
@@ -16295,10 +16295,10 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.3819</v>
+        <v>0.386</v>
       </c>
       <c r="G91" s="14" t="n">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H91" s="15" t="n">
         <v>100</v>
@@ -16325,7 +16325,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 38.2% (fair +162). Your call.</t>
+          <t>Model 38.6% (fair +159). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -16361,10 +16361,10 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.5332</v>
+        <v>0.5287999999999999</v>
       </c>
       <c r="G92" s="14" t="n">
-        <v>-114</v>
+        <v>-112</v>
       </c>
       <c r="H92" s="15" t="n">
         <v>117</v>
@@ -16391,7 +16391,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -16427,10 +16427,10 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.3459</v>
+        <v>0.3415</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="H93" s="15" t="n">
         <v>156</v>
@@ -16457,7 +16457,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 34.6% (fair +189). Your call.</t>
+          <t>Model 34.2% (fair +193). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -16493,10 +16493,10 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.6541</v>
+        <v>0.6585</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>-189</v>
+        <v>-193</v>
       </c>
       <c r="H94" s="15" t="n">
         <v>167</v>
@@ -16523,7 +16523,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 65.4% (fair -189). Your call.</t>
+          <t>Model 65.8% (fair -193). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -16559,10 +16559,10 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>0.4724</v>
+        <v>0.474</v>
       </c>
       <c r="G95" s="14" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H95" s="15" t="n">
         <v>104</v>
@@ -16589,7 +16589,7 @@
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>Model 47.2% (fair +112). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O95" s="15" t="n"/>
@@ -16625,13 +16625,13 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.5276</v>
+        <v>0.526</v>
       </c>
       <c r="G96" s="14" t="n">
-        <v>-112</v>
+        <v>-111</v>
       </c>
       <c r="H96" s="15" t="n">
-        <v>-106</v>
+        <v>-104</v>
       </c>
       <c r="I96" s="13">
         <f>IF($H$96="","",IF($H$96&lt;0,-$H$96/(-$H$96+100),100/($H$96+100)))</f>
@@ -16655,7 +16655,7 @@
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>Model 52.8% (fair -112). Your call.</t>
+          <t>Model 52.6% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O96" s="15" t="n"/>
@@ -16691,10 +16691,10 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.3115</v>
+        <v>0.3204</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="H97" s="15" t="n">
         <v>100</v>
@@ -16721,7 +16721,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 31.1% (fair +221). Your call.</t>
+          <t>Model 32.0% (fair +212). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16757,10 +16757,10 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.6089</v>
+        <v>0.5989</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>-156</v>
+        <v>-149</v>
       </c>
       <c r="H98" s="15" t="n">
         <v>117</v>
@@ -16787,7 +16787,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 59.9% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16823,10 +16823,10 @@
         </is>
       </c>
       <c r="F99" s="13" t="n">
-        <v>0.3614</v>
+        <v>0.3634</v>
       </c>
       <c r="G99" s="14" t="n">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H99" s="15" t="n">
         <v>156</v>
@@ -16853,7 +16853,7 @@
       </c>
       <c r="N99" s="19" t="inlineStr">
         <is>
-          <t>Model 36.1% (fair +177). Your call.</t>
+          <t>Model 36.3% (fair +175). Your call.</t>
         </is>
       </c>
       <c r="O99" s="15" t="n"/>
@@ -16889,10 +16889,10 @@
         </is>
       </c>
       <c r="F100" s="13" t="n">
-        <v>0.6386000000000001</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="G100" s="14" t="n">
-        <v>-177</v>
+        <v>-175</v>
       </c>
       <c r="H100" s="15" t="n">
         <v>167</v>
@@ -16919,7 +16919,7 @@
       </c>
       <c r="N100" s="19" t="inlineStr">
         <is>
-          <t>Model 63.9% (fair -177). Your call.</t>
+          <t>Model 63.7% (fair -175). Your call.</t>
         </is>
       </c>
       <c r="O100" s="15" t="n"/>
@@ -17351,7 +17351,7 @@
         </is>
       </c>
       <c r="F107" s="13" t="n">
-        <v>0.5071</v>
+        <v>0.5066999999999999</v>
       </c>
       <c r="G107" s="14" t="n">
         <v>-103</v>
@@ -17417,7 +17417,7 @@
         </is>
       </c>
       <c r="F108" s="13" t="n">
-        <v>0.4929</v>
+        <v>0.4933</v>
       </c>
       <c r="G108" s="14" t="n">
         <v>103</v>
@@ -17483,10 +17483,10 @@
         </is>
       </c>
       <c r="F109" s="13" t="n">
-        <v>0.462</v>
+        <v>0.4358</v>
       </c>
       <c r="G109" s="14" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="H109" s="15" t="n">
         <v>100</v>
@@ -17513,7 +17513,7 @@
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 43.6% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O109" s="15" t="n"/>
@@ -17549,10 +17549,10 @@
         </is>
       </c>
       <c r="F110" s="13" t="n">
-        <v>0.4508</v>
+        <v>0.4774</v>
       </c>
       <c r="G110" s="14" t="n">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="H110" s="15" t="n">
         <v>115</v>
@@ -17579,7 +17579,7 @@
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>Model 45.1% (fair +122). Your call.</t>
+          <t>Model 47.7% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O110" s="15" t="n"/>
@@ -17615,10 +17615,10 @@
         </is>
       </c>
       <c r="F111" s="13" t="n">
-        <v>0.5879</v>
+        <v>0.5935</v>
       </c>
       <c r="G111" s="14" t="n">
-        <v>-143</v>
+        <v>-146</v>
       </c>
       <c r="H111" s="15" t="n">
         <v>-143</v>
@@ -17645,7 +17645,7 @@
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -143). Your call.</t>
+          <t>Model 59.4% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O111" s="15" t="n"/>
@@ -17681,10 +17681,10 @@
         </is>
       </c>
       <c r="F112" s="13" t="n">
-        <v>0.4121</v>
+        <v>0.4065</v>
       </c>
       <c r="G112" s="14" t="n">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H112" s="15" t="n">
         <v>133</v>
@@ -17711,7 +17711,7 @@
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +143). Your call.</t>
+          <t>Model 40.6% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O112" s="15" t="n"/>
@@ -17747,13 +17747,13 @@
         </is>
       </c>
       <c r="F113" s="13" t="n">
-        <v>0.4685</v>
+        <v>0.4488576</v>
       </c>
       <c r="G113" s="14" t="n">
+        <v>123</v>
+      </c>
+      <c r="H113" s="15" t="n">
         <v>113</v>
-      </c>
-      <c r="H113" s="15" t="n">
-        <v>108</v>
       </c>
       <c r="I113" s="13">
         <f>IF($H$113="","",IF($H$113&lt;0,-$H$113/(-$H$113+100),100/($H$113+100)))</f>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="N113" s="19" t="inlineStr">
         <is>
-          <t>Model 46.9% (fair +113). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O113" s="15" t="n"/>
@@ -17813,13 +17813,13 @@
         </is>
       </c>
       <c r="F114" s="13" t="n">
-        <v>0.5315</v>
+        <v>0.5511424</v>
       </c>
       <c r="G114" s="14" t="n">
-        <v>-113</v>
+        <v>-123</v>
       </c>
       <c r="H114" s="15" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="I114" s="13">
         <f>IF($H$114="","",IF($H$114&lt;0,-$H$114/(-$H$114+100),100/($H$114+100)))</f>
@@ -17843,7 +17843,7 @@
       </c>
       <c r="N114" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O114" s="15" t="n"/>
@@ -17879,10 +17879,10 @@
         </is>
       </c>
       <c r="F115" s="13" t="n">
-        <v>0.5004999999999999</v>
+        <v>0.4851</v>
       </c>
       <c r="G115" s="14" t="n">
-        <v>-100</v>
+        <v>106</v>
       </c>
       <c r="H115" s="15" t="n">
         <v>105</v>
@@ -17909,7 +17909,7 @@
       </c>
       <c r="N115" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair -100). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O115" s="15" t="n"/>
@@ -17945,13 +17945,13 @@
         </is>
       </c>
       <c r="F116" s="13" t="n">
-        <v>0.4995000000000001</v>
+        <v>0.5149</v>
       </c>
       <c r="G116" s="14" t="n">
-        <v>100</v>
+        <v>-106</v>
       </c>
       <c r="H116" s="15" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="I116" s="13">
         <f>IF($H$116="","",IF($H$116&lt;0,-$H$116/(-$H$116+100),100/($H$116+100)))</f>
@@ -17975,7 +17975,7 @@
       </c>
       <c r="N116" s="19" t="inlineStr">
         <is>
-          <t>Model 50.0% (fair +100). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O116" s="15" t="n"/>
@@ -18011,10 +18011,10 @@
         </is>
       </c>
       <c r="F117" s="13" t="n">
-        <v>0.6162</v>
+        <v>0.6207</v>
       </c>
       <c r="G117" s="14" t="n">
-        <v>-161</v>
+        <v>-164</v>
       </c>
       <c r="H117" s="15" t="n">
         <v>-175</v>
@@ -18041,7 +18041,7 @@
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>Model 61.6% (fair -161). Your call.</t>
+          <t>Model 62.1% (fair -164). Your call.</t>
         </is>
       </c>
       <c r="O117" s="15" t="n"/>
@@ -18077,13 +18077,13 @@
         </is>
       </c>
       <c r="F118" s="13" t="n">
-        <v>0.3838</v>
+        <v>0.3793</v>
       </c>
       <c r="G118" s="14" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="H118" s="15" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I118" s="13">
         <f>IF($H$118="","",IF($H$118&lt;0,-$H$118/(-$H$118+100),100/($H$118+100)))</f>
@@ -18107,7 +18107,7 @@
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>Model 38.4% (fair +161). Your call.</t>
+          <t>Model 37.9% (fair +164). Your call.</t>
         </is>
       </c>
       <c r="O118" s="15" t="n"/>
@@ -18143,10 +18143,10 @@
         </is>
       </c>
       <c r="F119" s="13" t="n">
-        <v>0.5318000000000001</v>
+        <v>0.5354</v>
       </c>
       <c r="G119" s="14" t="n">
-        <v>-114</v>
+        <v>-115</v>
       </c>
       <c r="H119" s="15" t="n">
         <v>-113</v>
@@ -18173,7 +18173,7 @@
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 53.5% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O119" s="15" t="n"/>
@@ -18209,13 +18209,13 @@
         </is>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.4682</v>
+        <v>0.4646</v>
       </c>
       <c r="G120" s="14" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H120" s="15" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I120" s="13">
         <f>IF($H$120="","",IF($H$120&lt;0,-$H$120/(-$H$120+100),100/($H$120+100)))</f>
@@ -18239,7 +18239,7 @@
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 46.5% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O120" s="15" t="n"/>
@@ -18275,13 +18275,13 @@
         </is>
       </c>
       <c r="F121" s="13" t="n">
-        <v>0.5631</v>
+        <v>0.5516</v>
       </c>
       <c r="G121" s="14" t="n">
-        <v>-129</v>
+        <v>-123</v>
       </c>
       <c r="H121" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I121" s="13">
         <f>IF($H$121="","",IF($H$121&lt;0,-$H$121/(-$H$121+100),100/($H$121+100)))</f>
@@ -18305,7 +18305,7 @@
       </c>
       <c r="N121" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O121" s="15" t="n"/>
@@ -18341,10 +18341,10 @@
         </is>
       </c>
       <c r="F122" s="13" t="n">
-        <v>0.4369</v>
+        <v>0.4484</v>
       </c>
       <c r="G122" s="14" t="n">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H122" s="15" t="n">
         <v>100</v>
@@ -18371,7 +18371,7 @@
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O122" s="15" t="n"/>
@@ -18407,7 +18407,7 @@
         </is>
       </c>
       <c r="F123" s="13" t="n">
-        <v>0.5873</v>
+        <v>0.5865</v>
       </c>
       <c r="G123" s="14" t="n">
         <v>-142</v>
@@ -18473,7 +18473,7 @@
         </is>
       </c>
       <c r="F124" s="13" t="n">
-        <v>0.4127</v>
+        <v>0.4135</v>
       </c>
       <c r="G124" s="14" t="n">
         <v>142</v>
@@ -18539,10 +18539,10 @@
         </is>
       </c>
       <c r="F125" s="13" t="n">
-        <v>0.4843</v>
+        <v>0.4822</v>
       </c>
       <c r="G125" s="14" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H125" s="15" t="n">
         <v>108</v>
@@ -18569,7 +18569,7 @@
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +106). Your call.</t>
+          <t>Model 48.2% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O125" s="15" t="n"/>
@@ -18605,13 +18605,13 @@
         </is>
       </c>
       <c r="F126" s="13" t="n">
-        <v>0.5157</v>
+        <v>0.5178</v>
       </c>
       <c r="G126" s="14" t="n">
-        <v>-106</v>
+        <v>-107</v>
       </c>
       <c r="H126" s="15" t="n">
-        <v>-108</v>
+        <v>-111</v>
       </c>
       <c r="I126" s="13">
         <f>IF($H$126="","",IF($H$126&lt;0,-$H$126/(-$H$126+100),100/($H$126+100)))</f>
@@ -18635,7 +18635,7 @@
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -106). Your call.</t>
+          <t>Model 51.8% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O126" s="15" t="n"/>
@@ -18875,7 +18875,7 @@
         <v>-208</v>
       </c>
       <c r="H130" s="15" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I130" s="13">
         <f>IF($H$130="","",IF($H$130&lt;0,-$H$130/(-$H$130+100),100/($H$130+100)))</f>
@@ -19067,7 +19067,7 @@
         </is>
       </c>
       <c r="F133" s="13" t="n">
-        <v>0.5019</v>
+        <v>0.5032</v>
       </c>
       <c r="G133" s="14" t="n">
         <v>-101</v>
@@ -19097,7 +19097,7 @@
       </c>
       <c r="N133" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O133" s="15" t="n"/>
@@ -19133,7 +19133,7 @@
         </is>
       </c>
       <c r="F134" s="13" t="n">
-        <v>0.4981</v>
+        <v>0.4968</v>
       </c>
       <c r="G134" s="14" t="n">
         <v>101</v>
@@ -19163,7 +19163,7 @@
       </c>
       <c r="N134" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O134" s="15" t="n"/>
@@ -19199,10 +19199,10 @@
         </is>
       </c>
       <c r="F135" s="13" t="n">
-        <v>0.388</v>
+        <v>0.3915</v>
       </c>
       <c r="G135" s="14" t="n">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H135" s="15" t="n">
         <v>163</v>
@@ -19229,7 +19229,7 @@
       </c>
       <c r="N135" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 39.1% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O135" s="15" t="n"/>
@@ -19265,10 +19265,10 @@
         </is>
       </c>
       <c r="F136" s="13" t="n">
-        <v>0.612</v>
+        <v>0.6085</v>
       </c>
       <c r="G136" s="14" t="n">
-        <v>-158</v>
+        <v>-155</v>
       </c>
       <c r="H136" s="15" t="n">
         <v>-170</v>
@@ -19295,7 +19295,7 @@
       </c>
       <c r="N136" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 60.9% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O136" s="15" t="n"/>
@@ -19463,10 +19463,10 @@
         </is>
       </c>
       <c r="F139" s="13" t="n">
-        <v>0.5117</v>
+        <v>0.4961</v>
       </c>
       <c r="G139" s="14" t="n">
-        <v>-105</v>
+        <v>102</v>
       </c>
       <c r="H139" s="15" t="n">
         <v>108</v>
@@ -19493,7 +19493,7 @@
       </c>
       <c r="N139" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O139" s="15" t="n"/>
@@ -19529,13 +19529,13 @@
         </is>
       </c>
       <c r="F140" s="13" t="n">
-        <v>0.4883</v>
+        <v>0.5039</v>
       </c>
       <c r="G140" s="14" t="n">
-        <v>105</v>
+        <v>-102</v>
       </c>
       <c r="H140" s="15" t="n">
-        <v>105</v>
+        <v>-102</v>
       </c>
       <c r="I140" s="13">
         <f>IF($H$140="","",IF($H$140&lt;0,-$H$140/(-$H$140+100),100/($H$140+100)))</f>
@@ -19559,7 +19559,7 @@
       </c>
       <c r="N140" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O140" s="15" t="n"/>
@@ -19595,10 +19595,10 @@
         </is>
       </c>
       <c r="F141" s="13" t="n">
-        <v>0.3609</v>
+        <v>0.3618</v>
       </c>
       <c r="G141" s="14" t="n">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H141" s="15" t="n">
         <v>178</v>
@@ -19625,7 +19625,7 @@
       </c>
       <c r="N141" s="19" t="inlineStr">
         <is>
-          <t>Model 36.1% (fair +177). Your call.</t>
+          <t>Model 36.2% (fair +176). Your call.</t>
         </is>
       </c>
       <c r="O141" s="15" t="n"/>
@@ -19661,13 +19661,13 @@
         </is>
       </c>
       <c r="F142" s="13" t="n">
-        <v>0.6391</v>
+        <v>0.6382</v>
       </c>
       <c r="G142" s="14" t="n">
-        <v>-177</v>
+        <v>-176</v>
       </c>
       <c r="H142" s="15" t="n">
-        <v>-185</v>
+        <v>-182</v>
       </c>
       <c r="I142" s="13">
         <f>IF($H$142="","",IF($H$142&lt;0,-$H$142/(-$H$142+100),100/($H$142+100)))</f>
@@ -19691,7 +19691,7 @@
       </c>
       <c r="N142" s="19" t="inlineStr">
         <is>
-          <t>Model 63.9% (fair -177). Your call.</t>
+          <t>Model 63.8% (fair -176). Your call.</t>
         </is>
       </c>
       <c r="O142" s="15" t="n"/>
@@ -19859,13 +19859,13 @@
         </is>
       </c>
       <c r="F145" s="13" t="n">
-        <v>0.5494</v>
+        <v>0.646</v>
       </c>
       <c r="G145" s="14" t="n">
-        <v>-122</v>
+        <v>-182</v>
       </c>
       <c r="H145" s="15" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="I145" s="13">
         <f>IF($H$145="","",IF($H$145&lt;0,-$H$145/(-$H$145+100),100/($H$145+100)))</f>
@@ -19889,7 +19889,7 @@
       </c>
       <c r="N145" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 64.6% (fair -182). Your call.</t>
         </is>
       </c>
       <c r="O145" s="15" t="n"/>
@@ -19925,10 +19925,10 @@
         </is>
       </c>
       <c r="F146" s="13" t="n">
-        <v>0.4506</v>
+        <v>0.354</v>
       </c>
       <c r="G146" s="14" t="n">
-        <v>122</v>
+        <v>182</v>
       </c>
       <c r="H146" s="15" t="n">
         <v>100</v>
@@ -19955,7 +19955,7 @@
       </c>
       <c r="N146" s="19" t="inlineStr">
         <is>
-          <t>Model 45.1% (fair +122). Your call.</t>
+          <t>Model 35.4% (fair +182). Your call.</t>
         </is>
       </c>
       <c r="O146" s="15" t="n"/>
@@ -19991,10 +19991,10 @@
         </is>
       </c>
       <c r="F147" s="13" t="n">
-        <v>0.418</v>
+        <v>0.4169</v>
       </c>
       <c r="G147" s="14" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H147" s="15" t="n">
         <v>142</v>
@@ -20021,7 +20021,7 @@
       </c>
       <c r="N147" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 41.7% (fair +140). Your call.</t>
         </is>
       </c>
       <c r="O147" s="15" t="n"/>
@@ -20057,10 +20057,10 @@
         </is>
       </c>
       <c r="F148" s="13" t="n">
-        <v>0.5820000000000001</v>
+        <v>0.5831</v>
       </c>
       <c r="G148" s="14" t="n">
-        <v>-139</v>
+        <v>-140</v>
       </c>
       <c r="H148" s="15" t="n">
         <v>-145</v>
@@ -20087,7 +20087,7 @@
       </c>
       <c r="N148" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 58.3% (fair -140). Your call.</t>
         </is>
       </c>
       <c r="O148" s="15" t="n"/>
@@ -20123,7 +20123,7 @@
         </is>
       </c>
       <c r="F149" s="13" t="n">
-        <v>0.4592</v>
+        <v>0.4597</v>
       </c>
       <c r="G149" s="14" t="n">
         <v>118</v>
@@ -20151,7 +20151,7 @@
       </c>
       <c r="N149" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 46.0% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O149" s="15" t="n"/>
@@ -20187,7 +20187,7 @@
         </is>
       </c>
       <c r="F150" s="13" t="n">
-        <v>0.5407999999999999</v>
+        <v>0.5403</v>
       </c>
       <c r="G150" s="14" t="n">
         <v>-118</v>
@@ -20215,7 +20215,7 @@
       </c>
       <c r="N150" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O150" s="15" t="n"/>
@@ -20904,13 +20904,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4703000000000001</v>
+        <v>0.4641</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -20934,7 +20934,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 46.4% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -20970,13 +20970,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5296999999999999</v>
+        <v>0.5359</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -21000,7 +21000,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -21036,13 +21036,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5269667031772712</v>
+        <v>0.5202</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -21066,7 +21066,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -111). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -21102,13 +21102,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4730332968227288</v>
+        <v>0.4798</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -21132,7 +21132,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +111). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -21174,7 +21174,7 @@
         <v>-197</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -21240,7 +21240,7 @@
         <v>197</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -21306,7 +21306,7 @@
         <v>1157</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -21372,7 +21372,7 @@
         <v>-1157</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-115</v>
+        <v>-120</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -21432,13 +21432,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5867</v>
+        <v>0.5879</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-142</v>
+        <v>-143</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -21462,7 +21462,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 58.8% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -21498,10 +21498,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4133</v>
+        <v>0.4121</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>108</v>
@@ -21528,7 +21528,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 41.3% (fair +142). Your call.</t>
+          <t>Model 41.2% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -21570,7 +21570,7 @@
         <v>127</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -21636,7 +21636,7 @@
         <v>-112</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -21828,10 +21828,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5693</v>
+        <v>0.5705</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-132</v>
+        <v>-133</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>100</v>
@@ -21858,7 +21858,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -21894,13 +21894,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4307</v>
+        <v>0.4295</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-102</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -21924,7 +21924,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 43.0% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -21966,7 +21966,7 @@
         <v>-131</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -22616,14 +22616,14 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 180.5</t>
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5629</v>
+        <v>0.6194808686056472</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-129</v>
+        <v>-163</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>108</v>
@@ -22650,7 +22650,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 61.9% (fair -163). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -22682,17 +22682,17 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>Under 179.5</t>
+          <t>Under 180.5</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4371</v>
+        <v>0.3805191313943528</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>129</v>
+        <v>163</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>-105</v>
+        <v>104</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -22716,7 +22716,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 38.1% (fair +163). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -22752,13 +22752,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.4585</v>
+        <v>0.4597</v>
       </c>
       <c r="G33" s="14" t="n">
         <v>118</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>-106</v>
+        <v>-108</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -22782,7 +22782,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 46.0% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -22818,7 +22818,7 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5415</v>
+        <v>0.5403</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>-118</v>
@@ -22848,7 +22848,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -23016,10 +23016,10 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.5898</v>
+        <v>0.5886</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>-144</v>
+        <v>-143</v>
       </c>
       <c r="H37" s="15" t="n">
         <v>100</v>
@@ -23046,7 +23046,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -23082,13 +23082,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4102</v>
+        <v>0.4114</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -23112,7 +23112,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 41.0% (fair +144). Your call.</t>
+          <t>Model 41.1% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -23144,17 +23144,17 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury -4.5</t>
+          <t>Phoenix Mercury -3.5</t>
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.4602</v>
+        <v>0.4799</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>100</v>
+        <v>-105</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -23178,7 +23178,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -23210,17 +23210,17 @@
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>Connecticut Sun +4.5</t>
+          <t>Connecticut Sun +3.5</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5398000000000001</v>
+        <v>0.5201</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>-117</v>
+        <v>-108</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -23244,7 +23244,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -23359,28 +23359,28 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>0.2493</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>0.3914</v>
+        <v>0.3941</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>-95.11</v>
+        <v>-93.16</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>-14.15</v>
+        <v>-13.7</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>4.03</v>
+        <v>4.04</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>0.5406</v>
+        <v>0.5404</v>
       </c>
     </row>
     <row r="6">
@@ -23390,28 +23390,28 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>0.2498</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>603</v>
+        <v>611</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.3856</v>
+        <v>0.3888</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>-93.93000000000001</v>
+        <v>-91.97</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>-15.68</v>
+        <v>-15.15</v>
       </c>
       <c r="H6" s="24" t="n">
         <v>5.59</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>0.5581</v>
+        <v>0.5577</v>
       </c>
     </row>
     <row r="7">
@@ -23494,7 +23494,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>When the model said X%, how often it actually happened (n=440, ECE 0.052 — lower is better; a calibrated model's bars sit on the diagonal).</t>
+          <t>When the model said X%, how often it actually happened (n=443, ECE 0.051 — lower is better; a calibrated model's bars sit on the diagonal).</t>
         </is>
       </c>
     </row>
@@ -23570,16 +23570,16 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>0.3662</v>
+        <v>0.3667</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>0.5263</v>
+        <v>0.5385</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>0.1602</v>
+        <v>0.1718</v>
       </c>
     </row>
     <row r="20">
@@ -23608,16 +23608,16 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>0.543</v>
+        <v>0.5429</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.5306</v>
+        <v>0.533</v>
       </c>
       <c r="E21" s="26" t="n">
-        <v>-0.0124</v>
+        <v>-0.009900000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -23627,16 +23627,16 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>0.6401</v>
+        <v>0.6395</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0.5294</v>
+        <v>0.5385</v>
       </c>
       <c r="E22" s="27" t="n">
-        <v>-0.1106</v>
+        <v>-0.1011</v>
       </c>
     </row>
     <row r="23">

</xml_diff>